<commit_message>
feat: add data cleaning script and generate cleaned import data
</commit_message>
<xml_diff>
--- a/docs/data_cleaned.xlsx
+++ b/docs/data_cleaned.xlsx
@@ -30724,9 +30724,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="Q1103" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1104">
       <c r="A1104" t="n">
@@ -35161,9 +35158,6 @@
       <c r="Q1186" t="n">
         <v>9980</v>
       </c>
-      <c r="R1186" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1187">
       <c r="A1187" t="n">
@@ -35958,9 +35952,6 @@
       <c r="Q1199" t="n">
         <v>7000</v>
       </c>
-      <c r="R1199" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1200">
       <c r="A1200" t="n">
@@ -36020,9 +36011,6 @@
       <c r="Q1200" t="n">
         <v>5980</v>
       </c>
-      <c r="R1200" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1201">
       <c r="A1201" t="n">
@@ -36260,9 +36248,6 @@
       <c r="Q1204" t="n">
         <v>5980</v>
       </c>
-      <c r="R1204" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1205">
       <c r="A1205" t="n">
@@ -36753,9 +36738,6 @@
       <c r="Q1212" t="n">
         <v>9980</v>
       </c>
-      <c r="R1212" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1213">
       <c r="A1213" t="n">
@@ -37249,9 +37231,6 @@
       <c r="P1221" t="n">
         <v>5</v>
       </c>
-      <c r="R1221" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1222">
       <c r="A1222" t="n">
@@ -37978,12 +37957,6 @@
       <c r="P1234" t="n">
         <v>3</v>
       </c>
-      <c r="Q1234" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="R1234" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1235">
       <c r="A1235" t="n">
@@ -38043,9 +38016,6 @@
       <c r="Q1235" t="n">
         <v>4980</v>
       </c>
-      <c r="R1235" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1236">
       <c r="A1236" t="n">
@@ -38575,9 +38545,6 @@
       <c r="P1245" t="n">
         <v>1</v>
       </c>
-      <c r="R1245" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1246">
       <c r="A1246" t="n">
@@ -38629,12 +38596,6 @@
       <c r="P1246" t="n">
         <v>1</v>
       </c>
-      <c r="Q1246" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="R1246" t="e">
-        <v>#VALUE!</v>
-      </c>
     </row>
     <row r="1247">
       <c r="A1247" t="n">
@@ -39154,9 +39115,6 @@
       </c>
       <c r="P1256" t="n">
         <v>1</v>
-      </c>
-      <c r="R1256" t="e">
-        <v>#VALUE!</v>
       </c>
     </row>
     <row r="1257">

</xml_diff>

<commit_message>
fix: handle zero values in consume_level and numeric import fields
Root cause: Excel cells with 0 were imported as int, causing
asyncpg type mismatch (expected str, got int) for consume_level.

- clean_import_data.py: Convert 0 to None for consume_level,
  monthly_avg_shots, and monetary fields
- customers.py: Add backend protection for 0 → None conversion
</commit_message>
<xml_diff>
--- a/docs/data_cleaned.xlsx
+++ b/docs/data_cleaned.xlsx
@@ -31414,7 +31414,7 @@
         <v>4522</v>
       </c>
       <c r="P1126" t="n">
-        <v>4521.833333333333</v>
+        <v>4521</v>
       </c>
       <c r="Q1126" t="n">
         <v>678275</v>
@@ -31476,7 +31476,7 @@
         <v>4047</v>
       </c>
       <c r="P1127" t="n">
-        <v>4046.916666666667</v>
+        <v>4046</v>
       </c>
       <c r="Q1127" t="n">
         <v>631319</v>
@@ -31538,7 +31538,7 @@
         <v>3068</v>
       </c>
       <c r="P1128" t="n">
-        <v>3067.833333333333</v>
+        <v>3067</v>
       </c>
       <c r="Q1128" t="n">
         <v>294512</v>
@@ -31662,7 +31662,7 @@
         <v>2103</v>
       </c>
       <c r="P1130" t="n">
-        <v>2103.166666666667</v>
+        <v>2103</v>
       </c>
       <c r="Q1130" t="n">
         <v>353332</v>
@@ -31786,7 +31786,7 @@
         <v>1649</v>
       </c>
       <c r="P1132" t="n">
-        <v>1648.583333333333</v>
+        <v>1648</v>
       </c>
       <c r="Q1132" t="n">
         <v>197830</v>
@@ -31972,7 +31972,7 @@
         <v>1332</v>
       </c>
       <c r="P1135" t="n">
-        <v>1331.583333333333</v>
+        <v>1331</v>
       </c>
       <c r="Q1135" t="n">
         <v>183758.5</v>
@@ -32034,7 +32034,7 @@
         <v>1286</v>
       </c>
       <c r="P1136" t="n">
-        <v>1285.5</v>
+        <v>1285</v>
       </c>
       <c r="Q1136" t="n">
         <v>154260</v>
@@ -32158,7 +32158,7 @@
         <v>1211</v>
       </c>
       <c r="P1138" t="n">
-        <v>1210.666666666667</v>
+        <v>1210</v>
       </c>
       <c r="Q1138" t="n">
         <v>145280</v>
@@ -32220,7 +32220,7 @@
         <v>1167</v>
       </c>
       <c r="P1139" t="n">
-        <v>1167.083333333333</v>
+        <v>1167</v>
       </c>
       <c r="Q1139" t="n">
         <v>175062.5</v>
@@ -32282,7 +32282,7 @@
         <v>981</v>
       </c>
       <c r="P1140" t="n">
-        <v>980.5</v>
+        <v>980</v>
       </c>
       <c r="Q1140" t="n">
         <v>105894</v>
@@ -32406,7 +32406,7 @@
         <v>963</v>
       </c>
       <c r="P1142" t="n">
-        <v>962.6666666666666</v>
+        <v>962</v>
       </c>
       <c r="Q1142" t="n">
         <v>150176</v>
@@ -32468,7 +32468,7 @@
         <v>961</v>
       </c>
       <c r="P1143" t="n">
-        <v>960.8333333333334</v>
+        <v>960</v>
       </c>
       <c r="Q1143" t="n">
         <v>126830</v>
@@ -32530,7 +32530,7 @@
         <v>724</v>
       </c>
       <c r="P1144" t="n">
-        <v>723.9166666666666</v>
+        <v>723</v>
       </c>
       <c r="Q1144" t="n">
         <v>69496</v>
@@ -32597,7 +32597,7 @@
         <v>688</v>
       </c>
       <c r="P1145" t="n">
-        <v>687.5833333333334</v>
+        <v>687</v>
       </c>
       <c r="Q1145" t="n">
         <v>66008</v>
@@ -32659,7 +32659,7 @@
         <v>677</v>
       </c>
       <c r="P1146" t="n">
-        <v>676.5</v>
+        <v>676</v>
       </c>
       <c r="Q1146" t="n">
         <v>101475</v>
@@ -32721,7 +32721,7 @@
         <v>619</v>
       </c>
       <c r="P1147" t="n">
-        <v>618.6666666666666</v>
+        <v>618</v>
       </c>
       <c r="Q1147" t="n">
         <v>111360</v>
@@ -32907,7 +32907,7 @@
         <v>564</v>
       </c>
       <c r="P1150" t="n">
-        <v>564.3333333333334</v>
+        <v>564</v>
       </c>
       <c r="Q1150" t="n">
         <v>84650</v>
@@ -33157,7 +33157,7 @@
         <v>466</v>
       </c>
       <c r="P1154" t="n">
-        <v>466.3333333333333</v>
+        <v>466</v>
       </c>
       <c r="Q1154" t="n">
         <v>78344</v>
@@ -33348,7 +33348,7 @@
         <v>432</v>
       </c>
       <c r="P1157" t="n">
-        <v>431.5</v>
+        <v>431</v>
       </c>
       <c r="R1157" t="n">
         <v>70627.92</v>
@@ -33407,7 +33407,7 @@
         <v>430</v>
       </c>
       <c r="P1158" t="n">
-        <v>429.9166666666667</v>
+        <v>429</v>
       </c>
       <c r="Q1158" t="n">
         <v>64487.5</v>
@@ -33593,7 +33593,7 @@
         <v>411</v>
       </c>
       <c r="P1161" t="n">
-        <v>411.0833333333333</v>
+        <v>411</v>
       </c>
       <c r="Q1161" t="n">
         <v>73995</v>
@@ -33655,7 +33655,7 @@
         <v>338</v>
       </c>
       <c r="P1162" t="n">
-        <v>337.9166666666667</v>
+        <v>337</v>
       </c>
       <c r="Q1162" t="n">
         <v>60825</v>
@@ -33778,7 +33778,7 @@
         <v>287</v>
       </c>
       <c r="P1164" t="n">
-        <v>286.8333333333333</v>
+        <v>286</v>
       </c>
       <c r="Q1164" t="n">
         <v>41304</v>
@@ -33902,7 +33902,7 @@
         <v>249</v>
       </c>
       <c r="P1166" t="n">
-        <v>249.4166666666667</v>
+        <v>249</v>
       </c>
       <c r="Q1166" t="n">
         <v>44895</v>
@@ -34152,7 +34152,7 @@
         <v>172</v>
       </c>
       <c r="P1170" t="n">
-        <v>171.9166666666667</v>
+        <v>171</v>
       </c>
       <c r="Q1170" t="n">
         <v>16504</v>
@@ -34402,7 +34402,7 @@
         <v>145</v>
       </c>
       <c r="P1174" t="n">
-        <v>145.25</v>
+        <v>145</v>
       </c>
       <c r="Q1174" t="n">
         <v>13944</v>
@@ -34464,7 +34464,7 @@
         <v>143</v>
       </c>
       <c r="P1175" t="n">
-        <v>143.0833333333333</v>
+        <v>143</v>
       </c>
       <c r="Q1175" t="n">
         <v>13736</v>
@@ -34580,7 +34580,7 @@
         <v>125</v>
       </c>
       <c r="P1177" t="n">
-        <v>125.1666666666667</v>
+        <v>125</v>
       </c>
       <c r="Q1177" t="n">
         <v>22530</v>
@@ -34895,7 +34895,7 @@
         <v>78</v>
       </c>
       <c r="P1182" t="n">
-        <v>78.08333333333333</v>
+        <v>78</v>
       </c>
       <c r="Q1182" t="n">
         <v>14055</v>
@@ -35091,7 +35091,7 @@
         <v>61</v>
       </c>
       <c r="P1185" t="n">
-        <v>61.16666666666666</v>
+        <v>61</v>
       </c>
       <c r="Q1185" t="n">
         <v>5872</v>
@@ -35153,7 +35153,7 @@
         <v>59</v>
       </c>
       <c r="P1186" t="n">
-        <v>58.5</v>
+        <v>58</v>
       </c>
       <c r="Q1186" t="n">
         <v>9980</v>
@@ -35212,7 +35212,7 @@
         <v>57</v>
       </c>
       <c r="P1187" t="n">
-        <v>57.25</v>
+        <v>57</v>
       </c>
       <c r="Q1187" t="n">
         <v>6870</v>
@@ -35274,7 +35274,7 @@
         <v>55</v>
       </c>
       <c r="P1188" t="n">
-        <v>55.16666666666666</v>
+        <v>55</v>
       </c>
       <c r="Q1188" t="n">
         <v>9930</v>
@@ -35398,7 +35398,7 @@
         <v>45</v>
       </c>
       <c r="P1190" t="n">
-        <v>44.66666666666666</v>
+        <v>44</v>
       </c>
       <c r="Q1190" t="n">
         <v>26800</v>
@@ -35519,7 +35519,7 @@
         <v>42</v>
       </c>
       <c r="P1192" t="n">
-        <v>41.58333333333334</v>
+        <v>41</v>
       </c>
       <c r="Q1192" t="n">
         <v>6237.5</v>
@@ -35947,7 +35947,7 @@
         <v>29</v>
       </c>
       <c r="P1199" t="n">
-        <v>28.58333333333333</v>
+        <v>28</v>
       </c>
       <c r="Q1199" t="n">
         <v>7000</v>
@@ -36124,9 +36124,6 @@
       <c r="P1202" t="n">
         <v>28</v>
       </c>
-      <c r="R1202" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1203">
       <c r="A1203" t="n">
@@ -36181,7 +36178,7 @@
         <v>25</v>
       </c>
       <c r="P1203" t="n">
-        <v>25.33333333333333</v>
+        <v>25</v>
       </c>
       <c r="Q1203" t="n">
         <v>3040</v>
@@ -36299,9 +36296,6 @@
       <c r="P1205" t="n">
         <v>23</v>
       </c>
-      <c r="R1205" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1206">
       <c r="A1206" t="n">
@@ -36423,7 +36417,7 @@
         <v>21</v>
       </c>
       <c r="P1207" t="n">
-        <v>21.25</v>
+        <v>21</v>
       </c>
       <c r="Q1207" t="n">
         <v>6375</v>
@@ -36485,7 +36479,7 @@
         <v>21</v>
       </c>
       <c r="P1208" t="n">
-        <v>21.08333333333333</v>
+        <v>21</v>
       </c>
       <c r="Q1208" t="n">
         <v>3542</v>
@@ -36547,7 +36541,7 @@
         <v>18</v>
       </c>
       <c r="P1209" t="n">
-        <v>18.16666666666667</v>
+        <v>18</v>
       </c>
       <c r="Q1209" t="n">
         <v>4360</v>
@@ -36939,9 +36933,6 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="N1216" t="n">
-        <v>0</v>
-      </c>
       <c r="O1216" t="n">
         <v>8</v>
       </c>
@@ -37061,12 +37052,6 @@
       <c r="P1218" t="n">
         <v>7</v>
       </c>
-      <c r="Q1218" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1218" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1219">
       <c r="A1219" t="n">
@@ -37116,7 +37101,7 @@
         <v>6</v>
       </c>
       <c r="P1219" t="n">
-        <v>5.833333333333333</v>
+        <v>5</v>
       </c>
       <c r="Q1219" t="n">
         <v>6160</v>
@@ -37390,12 +37375,6 @@
       <c r="P1224" t="n">
         <v>4</v>
       </c>
-      <c r="Q1224" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1224" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1225">
       <c r="A1225" t="n">
@@ -37514,9 +37493,6 @@
       <c r="P1226" t="n">
         <v>4</v>
       </c>
-      <c r="R1226" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1227">
       <c r="A1227" t="n">
@@ -37673,12 +37649,6 @@
       <c r="P1229" t="n">
         <v>3</v>
       </c>
-      <c r="Q1229" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1229" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1230">
       <c r="A1230" t="n">
@@ -37838,12 +37808,6 @@
       <c r="P1232" t="n">
         <v>3</v>
       </c>
-      <c r="Q1232" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1232" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1233">
       <c r="A1233" t="n">
@@ -38174,12 +38138,6 @@
       <c r="P1238" t="n">
         <v>2</v>
       </c>
-      <c r="Q1238" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1238" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1239">
       <c r="A1239" t="n">
@@ -38334,12 +38292,6 @@
       <c r="P1241" t="n">
         <v>2</v>
       </c>
-      <c r="Q1241" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1241" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1242">
       <c r="A1242" t="n">
@@ -38647,9 +38599,6 @@
       <c r="P1247" t="n">
         <v>1</v>
       </c>
-      <c r="R1247" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1248">
       <c r="A1248" t="n">
@@ -38830,9 +38779,6 @@
       <c r="P1250" t="n">
         <v>1</v>
       </c>
-      <c r="R1250" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1251">
       <c r="A1251" t="n">
@@ -38884,9 +38830,6 @@
       <c r="P1251" t="n">
         <v>1</v>
       </c>
-      <c r="R1251" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1252">
       <c r="A1252" t="n">
@@ -38984,12 +38927,6 @@
       <c r="P1253" t="n">
         <v>1</v>
       </c>
-      <c r="Q1253" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1253" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1254">
       <c r="A1254" t="n">
@@ -39072,9 +39009,6 @@
       <c r="P1255" t="n">
         <v>1</v>
       </c>
-      <c r="R1255" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1256">
       <c r="A1256" t="n">
@@ -39280,12 +39214,6 @@
       <c r="P1259" t="n">
         <v>1</v>
       </c>
-      <c r="Q1259" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1259" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1260">
       <c r="A1260" t="n">
@@ -39337,12 +39265,6 @@
       <c r="P1260" t="n">
         <v>1</v>
       </c>
-      <c r="Q1260" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1260" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1261">
       <c r="A1261" t="n">
@@ -39496,12 +39418,6 @@
           <t>prepaid</t>
         </is>
       </c>
-      <c r="N1263" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1263" t="n">
-        <v>0</v>
-      </c>
       <c r="P1263" t="n">
         <v>1</v>
       </c>
@@ -39545,9 +39461,6 @@
           <t>C6</t>
         </is>
       </c>
-      <c r="O1264" t="n">
-        <v>0</v>
-      </c>
       <c r="P1264" t="n">
         <v>1</v>
       </c>
@@ -39591,15 +39504,6 @@
           <t>尽可能转Qverse，关停</t>
         </is>
       </c>
-      <c r="N1265" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1265" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1265" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1266">
       <c r="A1266" t="n">
@@ -39625,15 +39529,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1266" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1266" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1266" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1267">
       <c r="A1267" t="n">
@@ -39669,12 +39564,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1267" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1267" t="n">
-        <v>0</v>
-      </c>
       <c r="P1267" t="n">
         <v>7</v>
       </c>
@@ -39728,9 +39617,6 @@
           <t>C6</t>
         </is>
       </c>
-      <c r="O1268" t="n">
-        <v>0</v>
-      </c>
       <c r="P1268" t="n">
         <v>6</v>
       </c>
@@ -39774,9 +39660,6 @@
           <t>C6</t>
         </is>
       </c>
-      <c r="O1269" t="n">
-        <v>0</v>
-      </c>
       <c r="P1269" t="n">
         <v>2</v>
       </c>
@@ -39825,9 +39708,6 @@
           <t>C6</t>
         </is>
       </c>
-      <c r="O1270" t="n">
-        <v>0</v>
-      </c>
       <c r="P1270" t="n">
         <v>2</v>
       </c>
@@ -39866,15 +39746,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1271" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1271" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1271" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1272">
       <c r="A1272" t="n">
@@ -39900,15 +39771,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1272" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1272" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1272" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1273">
       <c r="A1273" t="n">
@@ -39939,15 +39801,6 @@
           <t>prepaid</t>
         </is>
       </c>
-      <c r="N1273" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1273" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1273" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1274">
       <c r="A1274" t="n">
@@ -39988,9 +39841,6 @@
           <t>C6</t>
         </is>
       </c>
-      <c r="O1274" t="n">
-        <v>0</v>
-      </c>
       <c r="P1274" t="n">
         <v>2</v>
       </c>
@@ -40034,12 +39884,6 @@
           <t>prepaid</t>
         </is>
       </c>
-      <c r="N1275" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1275" t="n">
-        <v>0</v>
-      </c>
       <c r="P1275" t="n">
         <v>22</v>
       </c>
@@ -40073,15 +39917,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1276" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1276" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1276" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1277">
       <c r="A1277" t="n">
@@ -40107,15 +39942,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1277" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1277" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1277" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1278">
       <c r="A1278" t="n">
@@ -40141,15 +39967,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1278" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1278" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1278" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1279">
       <c r="A1279" t="n">
@@ -40200,9 +40017,6 @@
           <t>C6</t>
         </is>
       </c>
-      <c r="O1279" t="n">
-        <v>0</v>
-      </c>
       <c r="P1279" t="n">
         <v>49</v>
       </c>
@@ -40231,15 +40045,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1280" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1280" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1280" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1281">
       <c r="A1281" t="n">
@@ -40265,15 +40070,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1281" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1281" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1281" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1282">
       <c r="A1282" t="n">
@@ -40304,15 +40100,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1282" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1282" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1282" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1283">
       <c r="A1283" t="n">
@@ -40338,15 +40125,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1283" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1283" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1283" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1284">
       <c r="A1284" t="n">
@@ -40387,9 +40165,6 @@
           <t>C6</t>
         </is>
       </c>
-      <c r="O1284" t="n">
-        <v>0</v>
-      </c>
       <c r="P1284" t="n">
         <v>2</v>
       </c>
@@ -40428,15 +40203,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1285" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1285" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1285" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1286">
       <c r="A1286" t="n">
@@ -40462,15 +40228,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1286" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1286" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1286" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1287">
       <c r="A1287" t="n">
@@ -40496,15 +40253,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1287" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1287" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1287" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1288">
       <c r="A1288" t="n">
@@ -40530,15 +40278,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1288" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1288" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1288" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1289">
       <c r="A1289" t="n">
@@ -40579,9 +40318,6 @@
           <t>C6</t>
         </is>
       </c>
-      <c r="O1289" t="n">
-        <v>0</v>
-      </c>
       <c r="P1289" t="n">
         <v>1</v>
       </c>
@@ -40610,15 +40346,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1290" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1290" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1290" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1291">
       <c r="A1291" t="n">
@@ -40644,15 +40371,6 @@
           <t>prepaid</t>
         </is>
       </c>
-      <c r="N1291" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1291" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1291" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1292">
       <c r="A1292" t="n">
@@ -40678,15 +40396,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1292" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1292" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1292" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1293">
       <c r="A1293" t="n">
@@ -40712,15 +40421,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1293" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1293" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1293" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1294">
       <c r="A1294" t="n">
@@ -40746,15 +40446,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1294" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1294" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1294" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1295">
       <c r="A1295" t="n">
@@ -40780,15 +40471,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1295" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1295" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1295" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1296">
       <c r="A1296" t="n">
@@ -40814,15 +40496,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1296" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1296" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1296" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1297">
       <c r="A1297" t="n">
@@ -40848,15 +40521,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1297" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1297" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1297" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1298">
       <c r="A1298" t="n">
@@ -40882,15 +40546,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1298" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1298" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1298" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1299">
       <c r="A1299" t="n">
@@ -40916,15 +40571,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1299" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1299" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1299" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1300">
       <c r="A1300" t="n">
@@ -40950,15 +40596,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1300" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1300" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1300" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1301">
       <c r="A1301" t="n">
@@ -40999,9 +40636,6 @@
           <t>C6</t>
         </is>
       </c>
-      <c r="O1301" t="n">
-        <v>0</v>
-      </c>
       <c r="P1301" t="n">
         <v>2</v>
       </c>
@@ -41030,15 +40664,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1302" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1302" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1302" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1303">
       <c r="A1303" t="n">
@@ -41064,15 +40689,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1303" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1303" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1303" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1304">
       <c r="A1304" t="n">
@@ -41093,15 +40709,6 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="N1304" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1304" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1304" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1305">
       <c r="A1305" t="n">
@@ -41127,15 +40734,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1305" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1305" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1305" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1306">
       <c r="A1306" t="n">
@@ -41161,15 +40759,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1306" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1306" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1306" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1307">
       <c r="A1307" t="n">
@@ -41200,15 +40789,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1307" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1307" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1307" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1308">
       <c r="A1308" t="n">
@@ -41239,15 +40819,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1308" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1308" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1308" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1309">
       <c r="A1309" t="n">
@@ -41273,15 +40844,6 @@
           <t>prepaid</t>
         </is>
       </c>
-      <c r="N1309" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1309" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1309" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1310">
       <c r="A1310" t="n">
@@ -41307,15 +40869,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1310" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1310" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1310" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1311">
       <c r="A1311" t="n">
@@ -41356,9 +40909,6 @@
           <t>C6</t>
         </is>
       </c>
-      <c r="O1311" t="n">
-        <v>0</v>
-      </c>
       <c r="P1311" t="n">
         <v>4</v>
       </c>
@@ -41382,15 +40932,6 @@
           <t>租房</t>
         </is>
       </c>
-      <c r="N1312" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1312" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1312" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1313">
       <c r="A1313" t="n">
@@ -41431,15 +40972,6 @@
           <t>prepaid</t>
         </is>
       </c>
-      <c r="N1313" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1313" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1313" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1314">
       <c r="A1314" t="n">
@@ -41460,15 +40992,6 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="N1314" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1314" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1314" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1315">
       <c r="A1315" t="n">
@@ -41489,15 +41012,6 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="N1315" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1315" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1315" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1316">
       <c r="A1316" t="n">
@@ -41528,15 +41042,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1316" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1316" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1316" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1317">
       <c r="A1317" t="n">
@@ -41567,15 +41072,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N1317" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1317" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1317" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1318">
       <c r="A1318" t="n">
@@ -41616,18 +41112,6 @@
           <t>prepaid</t>
         </is>
       </c>
-      <c r="O1318" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1318" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q1318" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1318" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1319">
       <c r="A1319" t="n">
@@ -41668,18 +41152,6 @@
           <t>prepaid</t>
         </is>
       </c>
-      <c r="O1319" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1319" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q1319" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1319" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1320">
       <c r="A1320" t="n">
@@ -41700,15 +41172,6 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="N1320" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1320" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1320" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1321">
       <c r="A1321" t="n">
@@ -41729,15 +41192,6 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="N1321" t="n">
-        <v>0</v>
-      </c>
-      <c r="O1321" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1321" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1322">
       <c r="A1322" t="n">
@@ -41778,18 +41232,6 @@
           <t>prepaid</t>
         </is>
       </c>
-      <c r="O1322" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1322" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q1322" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1322" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="1323">
       <c r="A1323" t="n">
@@ -41834,18 +41276,6 @@
         <is>
           <t>prepaid</t>
         </is>
-      </c>
-      <c r="O1323" t="n">
-        <v>0</v>
-      </c>
-      <c r="P1323" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q1323" t="n">
-        <v>0</v>
-      </c>
-      <c r="R1323" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="1324">

</xml_diff>